<commit_message>
Local uncommitted changes before rebase
</commit_message>
<xml_diff>
--- a/coin_data_template.xlsx
+++ b/coin_data_template.xlsx
@@ -436,7 +436,7 @@
         </is>
       </c>
       <c r="B1" s="3" t="n">
-        <v>45861</v>
+        <v>45866</v>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
@@ -460,12 +460,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>118160.72656250</t>
+          <t>118382.74218750</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>66674782208.00</t>
+          <t>61450612736.00</t>
         </is>
       </c>
     </row>
@@ -477,12 +477,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3588.97875977</t>
+          <t>3839.29833984</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40932126720.00</t>
+          <t>31396622336.00</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.13351941</t>
+          <t>3.18963933</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12542594048.00</t>
+          <t>7265161216.00</t>
         </is>
       </c>
     </row>
@@ -511,12 +511,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.00025249</t>
+          <t>0.99989623</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>141775290368.00</t>
+          <t>113312186368.00</t>
         </is>
       </c>
     </row>
@@ -528,12 +528,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>768.93322754</t>
+          <t>843.71435547</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4054797312.00</t>
+          <t>3934128640.00</t>
         </is>
       </c>
     </row>
@@ -545,12 +545,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>187.98310852</t>
+          <t>189.74516296</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>10916662272.00</t>
+          <t>6963974144.00</t>
         </is>
       </c>
     </row>
@@ -562,12 +562,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.99984008</t>
+          <t>0.99970394</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>16324828160.00</t>
+          <t>13242148864.00</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.23768300</t>
+          <t>0.23677585</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4269110016.00</t>
+          <t>2647860480.00</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.30729109</t>
+          <t>0.32443973</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1655781120.00</t>
+          <t>999039424.00</t>
         </is>
       </c>
     </row>
@@ -613,12 +613,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3570.79296875</t>
+          <t>3840.08154297</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>148800512.00</t>
+          <t>84654528.00</t>
         </is>
       </c>
     </row>
@@ -630,12 +630,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.80646747</t>
+          <t>0.81761342</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1937128576.00</t>
+          <t>1191408512.00</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>117959.80468750</t>
+          <t>118401.92968750</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>353885984.00</t>
+          <t>249355408.00</t>
         </is>
       </c>
     </row>
@@ -664,12 +664,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.42064092</t>
+          <t>0.43213448</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>909483776.00</t>
+          <t>414070496.00</t>
         </is>
       </c>
     </row>
@@ -681,12 +681,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4301.75244141</t>
+          <t>4656.18261719</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>15628827.00</t>
+          <t>5445967.00</t>
         </is>
       </c>
     </row>
@@ -698,12 +698,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>17.99403381</t>
+          <t>18.75102997</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>920663808.00</t>
+          <t>641334784.00</t>
         </is>
       </c>
     </row>
@@ -715,12 +715,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.24416417</t>
+          <t>0.27803397</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>703790464.00</t>
+          <t>633958272.00</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>508.21533203</t>
+          <t>581.97747803</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>551133632.00</t>
+          <t>832027648.00</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>23.71721458</t>
+          <t>26.79010963</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>906682688.00</t>
+          <t>1019868672.00</t>
         </is>
       </c>
     </row>
@@ -766,12 +766,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>8.96154785</t>
+          <t>8.96782398</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4582737.00</t>
+          <t>2473465.00</t>
         </is>
       </c>
     </row>
@@ -783,12 +783,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3808.16894531</t>
+          <t>4135.07275391</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>8637443.00</t>
+          <t>3981601.00</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.00001374</t>
+          <t>0.00001388</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>475206848.00</t>
+          <t>228340528.00</t>
         </is>
       </c>
     </row>
@@ -817,12 +817,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.20425153</t>
+          <t>3.34162569</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>336287.00</t>
+          <t>266564.00</t>
         </is>
       </c>
     </row>
@@ -834,12 +834,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3583.41235352</t>
+          <t>3853.48193359</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1783080704.00</t>
+          <t>1628264960.00</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>111.48131561</t>
+          <t>111.37905121</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1322818048.00</t>
+          <t>679937664.00</t>
         </is>
       </c>
     </row>
@@ -868,12 +868,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>43.87120819</t>
+          <t>44.25214767</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>76108504.00</t>
+          <t>64413124.00</t>
         </is>
       </c>
     </row>
@@ -885,12 +885,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>311.20404053</t>
+          <t>326.39016724</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>117212760.00</t>
+          <t>141200416.00</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4.09795761</t>
+          <t>4.15243149</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>533417792.00</t>
+          <t>276877536.00</t>
         </is>
       </c>
     </row>
@@ -919,12 +919,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.66845989</t>
+          <t>4.67224741</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>196493424.00</t>
+          <t>253308416.00</t>
         </is>
       </c>
     </row>
@@ -936,12 +936,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>288.29605103</t>
+          <t>297.28195190</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>659059776.00</t>
+          <t>423401344.00</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.99998087</t>
+          <t>0.99978793</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>22987296768.00</t>
+          <t>22449793024.00</t>
         </is>
       </c>
     </row>
@@ -970,12 +970,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.12048248</t>
+          <t>0.14222583</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>44030604.00</t>
+          <t>47653784.00</t>
         </is>
       </c>
     </row>
@@ -987,12 +987,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.07969487</t>
+          <t>1.13123858</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>145419184.00</t>
+          <t>135135936.00</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.18500257</t>
+          <t>1.18546247</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>15223631.00</t>
+          <t>17611844.00</t>
         </is>
       </c>
     </row>
@@ -1021,12 +1021,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2.74254537</t>
+          <t>2.88502860</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>317335040.00</t>
+          <t>242686240.00</t>
         </is>
       </c>
     </row>
@@ -1038,12 +1038,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.01767731</t>
+          <t>1.02975714</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>492531552.00</t>
+          <t>216409072.00</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5.54796457</t>
+          <t>5.77076530</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>133150904.00</t>
+          <t>110758976.00</t>
         </is>
       </c>
     </row>
@@ -1072,12 +1072,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>48.34008026</t>
+          <t>49.07056427</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>23989712.00</t>
+          <t>15563829.00</t>
         </is>
       </c>
     </row>
@@ -1089,12 +1089,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>228.97001648</t>
+          <t>231.36822510</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>56821368.00</t>
+          <t>32239178.00</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>22.39555931</t>
+          <t>22.53469849</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>320569088.00</t>
+          <t>211405136.00</t>
         </is>
       </c>
     </row>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.26463071</t>
+          <t>0.27390933</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>175466688.00</t>
+          <t>109012152.00</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.10362400</t>
+          <t>0.10163586</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>141669360.00</t>
+          <t>91356200.00</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.00003419</t>
+          <t>0.00003642</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1302272896.00</t>
+          <t>1124813696.00</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1174,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.45273060</t>
+          <t>0.65795863</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>680827200.00</t>
+          <t>1382552320.00</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0.02533145</t>
+          <t>0.02563172</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>84411136.00</t>
+          <t>47564300.00</t>
         </is>
       </c>
     </row>
@@ -1208,12 +1208,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>4.67824030</t>
+          <t>4.89323854</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>202652816.00</t>
+          <t>121866744.00</t>
         </is>
       </c>
     </row>
@@ -1242,12 +1242,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0.32917556</t>
+          <t>0.33718038</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>286890944.00</t>
+          <t>178097808.00</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>4.51130533</t>
+          <t>4.59706450</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>62996956.00</t>
+          <t>62431412.00</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1276,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>4.13666630</t>
+          <t>4.26197100</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>132999544.00</t>
+          <t>74641144.00</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>17.47446251</t>
+          <t>18.06102180</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>16744707.00</t>
+          <t>12238277.00</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.00076819</t>
+          <t>0.00082674</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>86.00</t>
+          <t>8.00</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.73909938</t>
+          <t>0.74463034</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>204704160.00</t>
+          <t>157006176.00</t>
         </is>
       </c>
     </row>
@@ -1344,12 +1344,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1.16557431</t>
+          <t>1.18790770</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>645574208.00</t>
+          <t>230530128.00</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1361,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2.62217665</t>
+          <t>2.72482228</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>340565664.00</t>
+          <t>190043568.00</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0.05325356</t>
+          <t>0.03714790</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.00</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1395,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>119.74081421</t>
+          <t>126.30731964</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>42349740.00</t>
+          <t>27688762.00</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1412,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>199.69749451</t>
+          <t>201.99955750</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>7733124.00</t>
+          <t>7382988.00</t>
         </is>
       </c>
     </row>
@@ -1429,12 +1429,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>5.07606983</t>
+          <t>5.12692833</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>33839248.00</t>
+          <t>28526776.00</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>0.00098251</t>
+          <t>0.00104364</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>352.00</t>
+          <t>10718.00</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>12.06196022</t>
+          <t>11.51330376</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>6182543.00</t>
+          <t>5720494.00</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.99814290</t>
+          <t>0.99819368</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>10459112448.00</t>
+          <t>6499842048.00</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>3750.54223633</t>
+          <t>4066.99902344</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>555469.00</t>
+          <t>169010.00</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>4058.71826172</t>
+          <t>4412.10498047</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>4752222.00</t>
+          <t>16496.00</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1.92223394</t>
+          <t>2.00494742</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>187665760.00</t>
+          <t>128772080.00</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>1.31564105</t>
+          <t>1.31532454</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>14184971.00</t>
+          <t>14968683.00</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>4.97862434</t>
+          <t>5.64388895</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>33674876.00</t>
+          <t>72850624.00</t>
         </is>
       </c>
     </row>
@@ -1582,12 +1582,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1.51207006</t>
+          <t>1.35311294</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>390288192.00</t>
+          <t>267781680.00</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1599,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>13.73220444</t>
+          <t>15.57480907</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>175816432.00</t>
+          <t>191689408.00</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.00001261</t>
+          <t>0.00001259</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>1492878592.00</t>
+          <t>928828160.00</t>
         </is>
       </c>
     </row>
@@ -1633,12 +1633,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.02286448</t>
+          <t>0.02437892</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>97335344.00</t>
+          <t>17261562.00</t>
         </is>
       </c>
     </row>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.08519785</t>
+          <t>0.09259591</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>58277992.00</t>
+          <t>50788068.00</t>
         </is>
       </c>
     </row>
@@ -1667,12 +1667,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.68822592</t>
+          <t>0.80022484</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>330961632.00</t>
+          <t>1055207104.00</t>
         </is>
       </c>
     </row>
@@ -1684,12 +1684,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>3747.10180664</t>
+          <t>4092.96044922</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>40637.00</t>
+          <t>65955.00</t>
         </is>
       </c>
     </row>
@@ -1701,12 +1701,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>117959.69531250</t>
+          <t>118398.72656250</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>1401545.00</t>
+          <t>396859.00</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1718,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>1.68242478</t>
+          <t>1.52858138</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>323265184.00</t>
+          <t>152509024.00</t>
         </is>
       </c>
     </row>
@@ -1735,12 +1735,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.79622054</t>
+          <t>0.80589938</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>370313824.00</t>
+          <t>259385376.00</t>
         </is>
       </c>
     </row>

</xml_diff>